<commit_message>
Deploying to gh-pages from @ eurovibes/rack-ser-adapter@1c3be01b343e4d63c33c68ce8a036fb5108c9a38 🚀
</commit_message>
<xml_diff>
--- a/Fabrication/BoM/rack-ser-adapter-bom_v0.1.xlsx
+++ b/Fabrication/BoM/rack-ser-adapter-bom_v0.1.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="49">
   <si>
     <t>Row</t>
   </si>
@@ -86,10 +86,10 @@
     <t>3</t>
   </si>
   <si>
-    <t>J1 J3</t>
-  </si>
-  <si>
-    <t>DB9_Female_MountingHoles</t>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>DE9_Pins_MountingHoles</t>
   </si>
   <si>
     <t>RS-232</t>
@@ -98,6 +98,15 @@
     <t>DSUB-9_Male_Horizontal_P2.77x2.84mm_EdgePinOffset4.94mm_Housed_MountingHolesOffset7.48mm</t>
   </si>
   <si>
+    <t>J3</t>
+  </si>
+  <si>
+    <t>DE9_Socket_MountingHoles</t>
+  </si>
+  <si>
+    <t>DSUB-9_Female_Horizontal_P2.77x2.84mm_EdgePinOffset4.94mm_Housed_MountingHolesOffset7.48mm</t>
+  </si>
+  <si>
     <t>KiBot Bill of Materials</t>
   </si>
   <si>
@@ -128,7 +137,7 @@
     <t>KiCad Version:</t>
   </si>
   <si>
-    <t>5.1.9+dfsg1-1~bpo10+1</t>
+    <t>10.0.5-unknown-202607221313~667fa36054~ubuntu25.10.1</t>
   </si>
   <si>
     <t>Component Groups:</t>
@@ -144,6 +153,9 @@
   </si>
   <si>
     <t>Total Components:</t>
+  </si>
+  <si>
+    <t>Columns colors</t>
   </si>
   <si>
     <t>KiCad Fields (default)</t>
@@ -256,34 +268,34 @@
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="justify" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="justify" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="justify" wrapText="1"/>
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="justify" wrapText="1"/>
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="justify" wrapText="1"/>
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="justify" wrapText="1"/>
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="justify" wrapText="1"/>
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="justify" wrapText="1"/>
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous" vertical="justify" wrapText="1"/>
+      <alignment horizontal="centerContinuous" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -296,7 +308,7 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
@@ -304,14 +316,23 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>995964</xdr:colOff>
-      <xdr:row>110</xdr:row>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>2977164</xdr:colOff>
+      <xdr:row>107</xdr:row>
       <xdr:rowOff>32809</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1" descr="logo.png"/>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+            <a:ext uri="{C183D7F6-B498-43B3-948B-1728B52AA6E4}">
+              <adec:decorative xmlns:adec="http://schemas.microsoft.com/office/drawing/2017/decorative" val="1"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -622,13 +643,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
     <col min="2" max="2" width="21.7109375" customWidth="1"/>
     <col min="3" max="3" width="29.7109375" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" customWidth="1"/>
+    <col min="4" max="4" width="52.7109375" customWidth="1"/>
     <col min="5" max="5" width="19.7109375" customWidth="1"/>
     <col min="6" max="6" width="20.7109375" customWidth="1"/>
     <col min="7" max="7" width="23.7109375" customWidth="1"/>
@@ -639,7 +660,7 @@
   <sheetData>
     <row r="1" spans="1:10" ht="32" customHeight="1">
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -651,27 +672,27 @@
     </row>
     <row r="2" spans="1:10">
       <c r="C2" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F2" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:10">
       <c r="C3" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F3" s="3">
         <v>8</v>
@@ -679,13 +700,13 @@
     </row>
     <row r="4" spans="1:10">
       <c r="C4" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="F4" s="3">
         <v>8</v>
@@ -693,13 +714,13 @@
     </row>
     <row r="5" spans="1:10">
       <c r="C5" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F5" s="3">
         <v>1</v>
@@ -707,13 +728,13 @@
     </row>
     <row r="6" spans="1:10">
       <c r="C6" s="2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F6" s="3">
         <v>8</v>
@@ -815,7 +836,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="30.0" customHeight="1">
+    <row r="11" spans="1:10" ht="45" customHeight="1">
       <c r="A11" s="5" t="s">
         <v>21</v>
       </c>
@@ -844,7 +865,39 @@
         <v>14</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>17</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="45" customHeight="1">
+      <c r="A12" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -855,34 +908,40 @@
     <hyperlink ref="G9" r:id="rId1"/>
     <hyperlink ref="G10" r:id="rId2"/>
     <hyperlink ref="G11" r:id="rId3"/>
+    <hyperlink ref="G12" r:id="rId4"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="50.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="6" t="s">
-        <v>42</v>
+      <c r="A1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:1">
-      <c r="A2" s="5" t="s">
-        <v>43</v>
+      <c r="A2" s="6" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" s="7" t="s">
-        <v>44</v>
+      <c r="A3" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="7" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>